<commit_message>
Use SofaScore as primary source for Phase 6 settlement
Flashscore upcoming feed drops finished matches; Phase 6 now queries
SofaScore last-events by team ID (from Phase 3) to get FT scores.
Flashscore feed retained as fallback. Settled today's 2 bets: both lost
(Everton 3-3 Man City, Sevilla 1-0 Real Sociedad).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase6_Settlement.xlsx
+++ b/docs/agent-system/outputs/Phase6_Settlement.xlsx
@@ -120,7 +120,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-05 01:28:49 ACST</t>
+          <t>2026-05-05 16:18:29 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -185,44 +185,44 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t/>
+          <t>3</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t/>
+          <t>3</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t/>
+          <t>draw</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>lost</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>-16.93</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Match status live; not yet settled.</t>
+          <t>[SofaScore] Pick home missed actual draw. Score 3-3.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-05 01:28:49 ACST</t>
+          <t>2026-05-05 16:18:29 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -287,37 +287,37 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t/>
+          <t>1</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t/>
+          <t>home</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>lost</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>-20.0</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Match status live; not yet settled.</t>
+          <t>[SofaScore] Pick away missed actual home. Score 1-0.</t>
         </is>
       </c>
     </row>
@@ -539,6 +539,210 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-05-05 16:18:29 ACST</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>flashscore:rTwrFuZR</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Premier League</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Everton</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Manchester City</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>0.2111</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>0.0573</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>16.93</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>bet</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>draw</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>lost</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>-16.93</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>[SofaScore] Pick home missed actual draw. Score 3-3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-05-05 16:18:29 ACST</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>flashscore:zs3PZaZa</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>LaLiga</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Sevilla</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Real Sociedad</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2.88</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>0.4819</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>0.1347</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>bet</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>lost</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>-20.0</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>[SofaScore] Pick away missed actual home. Score 1-0.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -648,210 +852,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-05-05 01:28:49 ACST</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>flashscore:rTwrFuZR</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Premier League</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>04:30</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Everton</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Manchester City</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>6.5</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>0.2111</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>0.0573</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>16.93</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>bet</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>Match status live; not yet settled.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-05-05 01:28:49 ACST</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>flashscore:zs3PZaZa</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>LaLiga</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>04:30</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Sevilla</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Real Sociedad</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>away</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2.88</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>0.4819</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>0.1347</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>bet</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>Match status live; not yet settled.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -879,7 +879,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -903,7 +903,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -927,7 +927,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>36.93</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-36.93</t>
         </is>
       </c>
     </row>
@@ -963,7 +963,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>-1.0</t>
         </is>
       </c>
     </row>
@@ -994,14 +994,14 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-05 01:28:49 ACST</t>
+          <t>2026-05-05 16:18:29 ACST</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>feed_health</t>
+          <t>sofa_health</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1013,55 +1013,55 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>feed_note</t>
+          <t>flashscore_health</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t/>
+          <t>healthy</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>phase5_input_rows</t>
+          <t>flashscore_note</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>rows_settled_this_run</t>
+          <t>phase5_input_rows</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>won_this_run</t>
+          <t>rows_settled_this_run</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>lost_this_run</t>
+          <t>won_this_run</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1073,7 +1073,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>lost_this_run</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1085,7 +1085,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>void</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>not_found</t>
+          <t>void</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1109,10 +1109,22 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>not_found</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>skipped</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>0</t>
         </is>

</xml_diff>